<commit_message>
ELV: ajuste em w.vel
</commit_message>
<xml_diff>
--- a/tabela de habitat.xlsx
+++ b/tabela de habitat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/480d9b848b88e342/MSS/_rebio23-mxr/mxr23_Q/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="11_E8FA0B9960DD2A79F7007CD708813A554CA11F24" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C49B060-9CE3-4541-97B1-5CFEBCB0E9F0}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_09FA781D42CFBA99372140D0B83CDD583E7D1A6F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6B82422-BFB9-42BE-AEFC-4956D10ACF0E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="279">
   <si>
     <t>Variable</t>
   </si>
@@ -332,6 +332,120 @@
     <t>3.7 (0-10)</t>
   </si>
   <si>
+    <t>14.6 (14.6-14.6)</t>
+  </si>
+  <si>
+    <t>80 (80-80)</t>
+  </si>
+  <si>
+    <t>16.7 (15-20)</t>
+  </si>
+  <si>
+    <t>Site 1</t>
+  </si>
+  <si>
+    <t>Site 2</t>
+  </si>
+  <si>
+    <t>Site 3</t>
+  </si>
+  <si>
+    <t>Site 4</t>
+  </si>
+  <si>
+    <t>Site 5</t>
+  </si>
+  <si>
+    <t>Site 6</t>
+  </si>
+  <si>
+    <t>Water quality</t>
+  </si>
+  <si>
+    <t>Dissolved oxigen (mg/L)</t>
+  </si>
+  <si>
+    <t>Conductivity (uS/cm)</t>
+  </si>
+  <si>
+    <t>Turbidity (NTU)</t>
+  </si>
+  <si>
+    <t>pH</t>
+  </si>
+  <si>
+    <t>Morphology</t>
+  </si>
+  <si>
+    <t>Elevation (m a.s.l.)</t>
+  </si>
+  <si>
+    <t>Water velocity (m/s)</t>
+  </si>
+  <si>
+    <t>Slope</t>
+  </si>
+  <si>
+    <t>Maximum depth (cm)</t>
+  </si>
+  <si>
+    <t>Average depth (cm)</t>
+  </si>
+  <si>
+    <t>Marginal depth (cm)</t>
+  </si>
+  <si>
+    <t>Width (m)</t>
+  </si>
+  <si>
+    <t>Substrate composition (%)</t>
+  </si>
+  <si>
+    <t>Mud</t>
+  </si>
+  <si>
+    <t>Sand</t>
+  </si>
+  <si>
+    <t>Habitat structures (%)</t>
+  </si>
+  <si>
+    <t>Aquatic macrophytes</t>
+  </si>
+  <si>
+    <t>Littoral grass</t>
+  </si>
+  <si>
+    <t>Submerged vegetation</t>
+  </si>
+  <si>
+    <t>Overhanging vegetation</t>
+  </si>
+  <si>
+    <t>Leaf litter</t>
+  </si>
+  <si>
+    <t>Fillamentous algae</t>
+  </si>
+  <si>
+    <t>Attached algae</t>
+  </si>
+  <si>
+    <t>Root masses</t>
+  </si>
+  <si>
+    <t>Small debris</t>
+  </si>
+  <si>
+    <t>Large debris</t>
+  </si>
+  <si>
+    <t>Temperature (°C)</t>
+  </si>
+  <si>
+    <t>7.0 (6.3-7.5)</t>
+  </si>
+  <si>
     <t>Variable</t>
   </si>
   <si>
@@ -482,15 +596,18 @@
     <t>m.Vel.m.s</t>
   </si>
   <si>
+    <t>0.017 (0-0.025)</t>
+  </si>
+  <si>
+    <t>0.035 (0.035-0.035)</t>
+  </si>
+  <si>
+    <t>0.073 (0.022-0.108)</t>
+  </si>
+  <si>
     <t>0 (0-0)</t>
   </si>
   <si>
-    <t>0.035 (0.035-0.035)</t>
-  </si>
-  <si>
-    <t>0.073 (0.022-0.108)</t>
-  </si>
-  <si>
     <t>0.293 (0.25-0.348)</t>
   </si>
   <si>
@@ -590,6 +707,9 @@
     <t>1.7 (1.1-2.1)</t>
   </si>
   <si>
+    <t>14.6 (14.6-14.6)</t>
+  </si>
+  <si>
     <t>1.2 (0.8-1.6)</t>
   </si>
   <si>
@@ -605,6 +725,9 @@
     <t>90 (90-90)</t>
   </si>
   <si>
+    <t>80 (80-80)</t>
+  </si>
+  <si>
     <t>70 (60-80)</t>
   </si>
   <si>
@@ -710,6 +833,9 @@
     <t>2.3 (1-5)</t>
   </si>
   <si>
+    <t>16.7 (15-20)</t>
+  </si>
+  <si>
     <t>h.Root.masses</t>
   </si>
   <si>
@@ -732,136 +858,16 @@
   </si>
   <si>
     <t>3.7 (0-10)</t>
-  </si>
-  <si>
-    <t>14.6 (14.6-14.6)</t>
-  </si>
-  <si>
-    <t>80 (80-80)</t>
-  </si>
-  <si>
-    <t>16.7 (15-20)</t>
-  </si>
-  <si>
-    <t>Site 1</t>
-  </si>
-  <si>
-    <t>Site 2</t>
-  </si>
-  <si>
-    <t>Site 3</t>
-  </si>
-  <si>
-    <t>Site 4</t>
-  </si>
-  <si>
-    <t>Site 5</t>
-  </si>
-  <si>
-    <t>Site 6</t>
-  </si>
-  <si>
-    <t>Water quality</t>
-  </si>
-  <si>
-    <t>Dissolved oxigen (mg/L)</t>
-  </si>
-  <si>
-    <t>Conductivity (uS/cm)</t>
-  </si>
-  <si>
-    <t>Turbidity (NTU)</t>
-  </si>
-  <si>
-    <t>pH</t>
-  </si>
-  <si>
-    <t>Morphology</t>
-  </si>
-  <si>
-    <t>Elevation (m a.s.l.)</t>
-  </si>
-  <si>
-    <t>Water velocity (m/s)</t>
-  </si>
-  <si>
-    <t>Slope</t>
-  </si>
-  <si>
-    <t>Maximum depth (cm)</t>
-  </si>
-  <si>
-    <t>Average depth (cm)</t>
-  </si>
-  <si>
-    <t>Marginal depth (cm)</t>
-  </si>
-  <si>
-    <t>Width (m)</t>
-  </si>
-  <si>
-    <t>Substrate composition (%)</t>
-  </si>
-  <si>
-    <t>Mud</t>
-  </si>
-  <si>
-    <t>Sand</t>
-  </si>
-  <si>
-    <t>Habitat structures (%)</t>
-  </si>
-  <si>
-    <t>Aquatic macrophytes</t>
-  </si>
-  <si>
-    <t>Littoral grass</t>
-  </si>
-  <si>
-    <t>Submerged vegetation</t>
-  </si>
-  <si>
-    <t>Overhanging vegetation</t>
-  </si>
-  <si>
-    <t>Leaf litter</t>
-  </si>
-  <si>
-    <t>Fillamentous algae</t>
-  </si>
-  <si>
-    <t>Attached algae</t>
-  </si>
-  <si>
-    <t>Root masses</t>
-  </si>
-  <si>
-    <t>Small debris</t>
-  </si>
-  <si>
-    <t>Large debris</t>
-  </si>
-  <si>
-    <t>Temperature (°C)</t>
-  </si>
-  <si>
-    <t>7.0 (6.3-7.5)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -904,10 +910,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1194,577 +1196,577 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>103</v>
+        <v>141</v>
       </c>
       <c r="B1" t="s">
-        <v>104</v>
+        <v>142</v>
       </c>
       <c r="C1" t="s">
-        <v>105</v>
+        <v>143</v>
       </c>
       <c r="D1" t="s">
-        <v>106</v>
+        <v>144</v>
       </c>
       <c r="E1" t="s">
-        <v>107</v>
+        <v>145</v>
       </c>
       <c r="F1" t="s">
-        <v>108</v>
+        <v>146</v>
       </c>
       <c r="G1" t="s">
-        <v>109</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>110</v>
+        <v>148</v>
       </c>
       <c r="B2" t="s">
-        <v>111</v>
+        <v>149</v>
       </c>
       <c r="C2" t="s">
-        <v>112</v>
+        <v>150</v>
       </c>
       <c r="D2" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="E2" t="s">
-        <v>114</v>
+        <v>152</v>
       </c>
       <c r="F2" t="s">
-        <v>115</v>
+        <v>153</v>
       </c>
       <c r="G2" t="s">
-        <v>116</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>117</v>
+        <v>155</v>
       </c>
       <c r="B3" t="s">
-        <v>118</v>
+        <v>156</v>
       </c>
       <c r="C3" t="s">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="D3" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="E3" t="s">
-        <v>121</v>
+        <v>159</v>
       </c>
       <c r="F3" t="s">
-        <v>122</v>
+        <v>160</v>
       </c>
       <c r="G3" t="s">
-        <v>123</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>124</v>
+        <v>162</v>
       </c>
       <c r="B4" t="s">
-        <v>125</v>
+        <v>163</v>
       </c>
       <c r="C4" t="s">
-        <v>126</v>
+        <v>164</v>
       </c>
       <c r="D4" t="s">
-        <v>127</v>
+        <v>165</v>
       </c>
       <c r="E4" t="s">
-        <v>128</v>
+        <v>166</v>
       </c>
       <c r="F4" t="s">
-        <v>129</v>
+        <v>167</v>
       </c>
       <c r="G4" t="s">
-        <v>130</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>131</v>
+        <v>169</v>
       </c>
       <c r="B5" t="s">
-        <v>132</v>
+        <v>170</v>
       </c>
       <c r="C5" t="s">
-        <v>133</v>
+        <v>171</v>
       </c>
       <c r="D5" t="s">
-        <v>134</v>
+        <v>172</v>
       </c>
       <c r="E5" t="s">
-        <v>135</v>
+        <v>173</v>
       </c>
       <c r="F5" t="s">
-        <v>136</v>
+        <v>174</v>
       </c>
       <c r="G5" t="s">
-        <v>137</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>138</v>
+        <v>176</v>
       </c>
       <c r="B6" t="s">
-        <v>139</v>
+        <v>177</v>
       </c>
       <c r="C6" t="s">
-        <v>140</v>
+        <v>178</v>
       </c>
       <c r="D6" t="s">
-        <v>141</v>
+        <v>179</v>
       </c>
       <c r="E6" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="F6" t="s">
-        <v>143</v>
+        <v>181</v>
       </c>
       <c r="G6" t="s">
-        <v>144</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>145</v>
+        <v>183</v>
       </c>
       <c r="B7" t="s">
-        <v>146</v>
+        <v>184</v>
       </c>
       <c r="C7" t="s">
-        <v>147</v>
+        <v>185</v>
       </c>
       <c r="D7" t="s">
-        <v>148</v>
+        <v>186</v>
       </c>
       <c r="E7" t="s">
-        <v>149</v>
+        <v>187</v>
       </c>
       <c r="F7" t="s">
-        <v>150</v>
+        <v>188</v>
       </c>
       <c r="G7" t="s">
-        <v>151</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>152</v>
+        <v>190</v>
       </c>
       <c r="B8" t="s">
-        <v>153</v>
+        <v>191</v>
       </c>
       <c r="C8" t="s">
-        <v>154</v>
+        <v>192</v>
       </c>
       <c r="D8" t="s">
-        <v>155</v>
+        <v>193</v>
       </c>
       <c r="E8" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="F8" t="s">
-        <v>156</v>
+        <v>195</v>
       </c>
       <c r="G8" t="s">
-        <v>157</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>158</v>
+        <v>197</v>
       </c>
       <c r="B9" t="s">
-        <v>159</v>
+        <v>198</v>
       </c>
       <c r="C9" t="s">
-        <v>160</v>
+        <v>199</v>
       </c>
       <c r="D9" t="s">
-        <v>161</v>
+        <v>200</v>
       </c>
       <c r="E9" t="s">
-        <v>162</v>
+        <v>201</v>
       </c>
       <c r="F9" t="s">
-        <v>163</v>
+        <v>202</v>
       </c>
       <c r="G9" t="s">
-        <v>164</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>165</v>
+        <v>204</v>
       </c>
       <c r="B10" t="s">
-        <v>166</v>
+        <v>205</v>
       </c>
       <c r="C10" t="s">
-        <v>167</v>
+        <v>206</v>
       </c>
       <c r="D10" t="s">
-        <v>168</v>
+        <v>207</v>
       </c>
       <c r="E10" t="s">
-        <v>169</v>
+        <v>208</v>
       </c>
       <c r="F10" t="s">
-        <v>170</v>
+        <v>209</v>
       </c>
       <c r="G10" t="s">
-        <v>171</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>172</v>
+        <v>211</v>
       </c>
       <c r="B11" t="s">
-        <v>173</v>
+        <v>212</v>
       </c>
       <c r="C11" t="s">
-        <v>174</v>
+        <v>213</v>
       </c>
       <c r="D11" t="s">
-        <v>175</v>
+        <v>214</v>
       </c>
       <c r="E11" t="s">
-        <v>176</v>
+        <v>215</v>
       </c>
       <c r="F11" t="s">
-        <v>177</v>
+        <v>216</v>
       </c>
       <c r="G11" t="s">
-        <v>178</v>
+        <v>217</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>179</v>
+        <v>218</v>
       </c>
       <c r="B12" t="s">
-        <v>166</v>
+        <v>205</v>
       </c>
       <c r="C12" t="s">
-        <v>180</v>
+        <v>219</v>
       </c>
       <c r="D12" t="s">
-        <v>181</v>
+        <v>220</v>
       </c>
       <c r="E12" t="s">
-        <v>182</v>
+        <v>221</v>
       </c>
       <c r="F12" t="s">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="G12" t="s">
-        <v>184</v>
+        <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>185</v>
+        <v>224</v>
       </c>
       <c r="B13" t="s">
-        <v>186</v>
+        <v>225</v>
       </c>
       <c r="C13" t="s">
-        <v>187</v>
+        <v>226</v>
       </c>
       <c r="D13" t="s">
-        <v>188</v>
+        <v>227</v>
       </c>
       <c r="E13" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="F13" t="s">
-        <v>189</v>
+        <v>229</v>
       </c>
       <c r="G13" t="s">
-        <v>190</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>191</v>
+        <v>231</v>
       </c>
       <c r="B14" t="s">
-        <v>192</v>
+        <v>232</v>
       </c>
       <c r="C14" t="s">
-        <v>192</v>
+        <v>232</v>
       </c>
       <c r="D14" t="s">
-        <v>193</v>
+        <v>233</v>
       </c>
       <c r="E14" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="F14" t="s">
-        <v>194</v>
+        <v>235</v>
       </c>
       <c r="G14" t="s">
-        <v>195</v>
+        <v>236</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>196</v>
+        <v>237</v>
       </c>
       <c r="B15" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="C15" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="D15" t="s">
-        <v>197</v>
+        <v>238</v>
       </c>
       <c r="E15" t="s">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="F15" t="s">
-        <v>198</v>
+        <v>239</v>
       </c>
       <c r="G15" t="s">
-        <v>199</v>
+        <v>240</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>200</v>
+        <v>241</v>
       </c>
       <c r="B16" t="s">
-        <v>201</v>
+        <v>242</v>
       </c>
       <c r="C16" t="s">
-        <v>202</v>
+        <v>243</v>
       </c>
       <c r="D16" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="E16" t="s">
-        <v>203</v>
+        <v>244</v>
       </c>
       <c r="F16" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="G16" t="s">
-        <v>204</v>
+        <v>245</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>205</v>
+        <v>246</v>
       </c>
       <c r="B17" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="C17" t="s">
-        <v>201</v>
+        <v>242</v>
       </c>
       <c r="D17" t="s">
-        <v>206</v>
+        <v>247</v>
       </c>
       <c r="E17" t="s">
-        <v>207</v>
+        <v>248</v>
       </c>
       <c r="F17" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="G17" t="s">
-        <v>208</v>
+        <v>249</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>209</v>
+        <v>250</v>
       </c>
       <c r="B18" t="s">
-        <v>201</v>
+        <v>242</v>
       </c>
       <c r="C18" t="s">
-        <v>210</v>
+        <v>251</v>
       </c>
       <c r="D18" t="s">
-        <v>211</v>
+        <v>252</v>
       </c>
       <c r="E18" t="s">
-        <v>212</v>
+        <v>253</v>
       </c>
       <c r="F18" t="s">
-        <v>213</v>
+        <v>254</v>
       </c>
       <c r="G18" t="s">
-        <v>214</v>
+        <v>255</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>215</v>
+        <v>256</v>
       </c>
       <c r="B19" t="s">
-        <v>193</v>
+        <v>233</v>
       </c>
       <c r="C19" t="s">
-        <v>216</v>
+        <v>257</v>
       </c>
       <c r="D19" t="s">
-        <v>217</v>
+        <v>258</v>
       </c>
       <c r="E19" t="s">
-        <v>180</v>
+        <v>219</v>
       </c>
       <c r="F19" t="s">
-        <v>194</v>
+        <v>235</v>
       </c>
       <c r="G19" t="s">
-        <v>218</v>
+        <v>259</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>219</v>
+        <v>260</v>
       </c>
       <c r="B20" t="s">
-        <v>197</v>
+        <v>238</v>
       </c>
       <c r="C20" t="s">
-        <v>220</v>
+        <v>261</v>
       </c>
       <c r="D20" t="s">
-        <v>221</v>
+        <v>262</v>
       </c>
       <c r="E20" t="s">
-        <v>222</v>
+        <v>263</v>
       </c>
       <c r="F20" t="s">
-        <v>208</v>
+        <v>249</v>
       </c>
       <c r="G20" t="s">
-        <v>223</v>
+        <v>264</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>224</v>
+        <v>265</v>
       </c>
       <c r="B21" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="C21" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="D21" t="s">
-        <v>225</v>
+        <v>266</v>
       </c>
       <c r="E21" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="F21" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="G21" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>226</v>
+        <v>267</v>
       </c>
       <c r="B22" t="s">
-        <v>201</v>
+        <v>242</v>
       </c>
       <c r="C22" t="s">
-        <v>227</v>
+        <v>268</v>
       </c>
       <c r="D22" t="s">
-        <v>228</v>
+        <v>269</v>
       </c>
       <c r="E22" t="s">
-        <v>239</v>
+        <v>270</v>
       </c>
       <c r="F22" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="G22" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>229</v>
+        <v>271</v>
       </c>
       <c r="B23" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="C23" t="s">
-        <v>210</v>
+        <v>251</v>
       </c>
       <c r="D23" t="s">
-        <v>230</v>
+        <v>272</v>
       </c>
       <c r="E23" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="F23" t="s">
-        <v>231</v>
+        <v>273</v>
       </c>
       <c r="G23" t="s">
-        <v>211</v>
+        <v>252</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>232</v>
+        <v>274</v>
       </c>
       <c r="B24" t="s">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="C24" t="s">
-        <v>227</v>
+        <v>268</v>
       </c>
       <c r="D24" t="s">
-        <v>233</v>
+        <v>275</v>
       </c>
       <c r="E24" t="s">
-        <v>234</v>
+        <v>276</v>
       </c>
       <c r="F24" t="s">
-        <v>211</v>
+        <v>252</v>
       </c>
       <c r="G24" t="s">
-        <v>201</v>
+        <v>242</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>235</v>
+        <v>277</v>
       </c>
       <c r="B25" t="s">
-        <v>197</v>
+        <v>238</v>
       </c>
       <c r="C25" t="s">
-        <v>201</v>
+        <v>242</v>
       </c>
       <c r="D25" t="s">
-        <v>236</v>
+        <v>278</v>
       </c>
       <c r="E25" t="s">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="F25" t="s">
-        <v>208</v>
+        <v>249</v>
       </c>
       <c r="G25" t="s">
-        <v>230</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -1783,32 +1785,32 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>240</v>
+        <v>106</v>
       </c>
       <c r="C1" t="s">
-        <v>241</v>
+        <v>107</v>
       </c>
       <c r="D1" t="s">
-        <v>242</v>
+        <v>108</v>
       </c>
       <c r="E1" t="s">
-        <v>243</v>
+        <v>109</v>
       </c>
       <c r="F1" t="s">
-        <v>244</v>
+        <v>110</v>
       </c>
       <c r="G1" t="s">
-        <v>245</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>246</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>273</v>
+        <v>139</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
@@ -1831,7 +1833,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>247</v>
+        <v>113</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
@@ -1854,7 +1856,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>248</v>
+        <v>114</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
@@ -1877,7 +1879,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>249</v>
+        <v>115</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
@@ -1900,10 +1902,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>250</v>
+        <v>116</v>
       </c>
       <c r="B7" t="s">
-        <v>274</v>
+        <v>140</v>
       </c>
       <c r="C7" t="s">
         <v>25</v>
@@ -1923,12 +1925,12 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>251</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>252</v>
+        <v>118</v>
       </c>
       <c r="B9" t="s">
         <v>30</v>
@@ -1951,7 +1953,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>258</v>
+        <v>124</v>
       </c>
       <c r="B10" t="s">
         <v>64</v>
@@ -1963,7 +1965,7 @@
         <v>66</v>
       </c>
       <c r="E10" t="s">
-        <v>237</v>
+        <v>103</v>
       </c>
       <c r="F10" t="s">
         <v>67</v>
@@ -1974,10 +1976,10 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>253</v>
+        <v>119</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>191</v>
       </c>
       <c r="C11" t="s">
         <v>37</v>
@@ -1997,7 +1999,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>254</v>
+        <v>120</v>
       </c>
       <c r="B12" t="s">
         <v>41</v>
@@ -2020,7 +2022,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>255</v>
+        <v>121</v>
       </c>
       <c r="B13" t="s">
         <v>47</v>
@@ -2043,7 +2045,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>256</v>
+        <v>122</v>
       </c>
       <c r="B14" t="s">
         <v>53</v>
@@ -2066,7 +2068,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>257</v>
+        <v>123</v>
       </c>
       <c r="B15" t="s">
         <v>47</v>
@@ -2089,12 +2091,12 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>259</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>260</v>
+        <v>126</v>
       </c>
       <c r="B17" t="s">
         <v>69</v>
@@ -2106,7 +2108,7 @@
         <v>70</v>
       </c>
       <c r="E17" t="s">
-        <v>238</v>
+        <v>104</v>
       </c>
       <c r="F17" t="s">
         <v>71</v>
@@ -2117,7 +2119,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>261</v>
+        <v>127</v>
       </c>
       <c r="B18" t="s">
         <v>36</v>
@@ -2140,12 +2142,12 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>262</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>263</v>
+        <v>129</v>
       </c>
       <c r="B20" t="s">
         <v>76</v>
@@ -2168,7 +2170,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>264</v>
+        <v>130</v>
       </c>
       <c r="B21" t="s">
         <v>36</v>
@@ -2191,7 +2193,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>265</v>
+        <v>131</v>
       </c>
       <c r="B22" t="s">
         <v>76</v>
@@ -2214,7 +2216,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>266</v>
+        <v>132</v>
       </c>
       <c r="B23" t="s">
         <v>70</v>
@@ -2237,7 +2239,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>267</v>
+        <v>133</v>
       </c>
       <c r="B24" t="s">
         <v>73</v>
@@ -2260,7 +2262,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>268</v>
+        <v>134</v>
       </c>
       <c r="B25" t="s">
         <v>36</v>
@@ -2283,7 +2285,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>269</v>
+        <v>135</v>
       </c>
       <c r="B26" t="s">
         <v>76</v>
@@ -2295,7 +2297,7 @@
         <v>97</v>
       </c>
       <c r="E26" t="s">
-        <v>239</v>
+        <v>105</v>
       </c>
       <c r="F26" t="s">
         <v>36</v>
@@ -2306,7 +2308,7 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>272</v>
+        <v>138</v>
       </c>
       <c r="B27" t="s">
         <v>62</v>
@@ -2329,7 +2331,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>271</v>
+        <v>137</v>
       </c>
       <c r="B28" t="s">
         <v>73</v>
@@ -2352,7 +2354,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>270</v>
+        <v>136</v>
       </c>
       <c r="B29" t="s">
         <v>36</v>
@@ -2374,7 +2376,6 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
ELV: sem erro no arquivo RDS
</commit_message>
<xml_diff>
--- a/tabela de habitat.xlsx
+++ b/tabela de habitat.xlsx
@@ -1,27 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="tabela_final" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="tabela_final" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="156">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
@@ -494,11 +488,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -507,26 +501,10 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -538,7 +516,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -546,49 +524,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="left" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
 </styleSheet>
 </file>
 
@@ -768,1056 +717,1055 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G1048576"/>
-  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" t="s">
         <v>40</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" t="s">
         <v>43</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" t="s">
         <v>46</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="F7" t="s">
         <v>47</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="G7" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" t="s">
         <v>51</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" t="s">
         <v>52</v>
       </c>
-      <c r="E8" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="F8" s="0" t="s">
+      <c r="E8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" t="s">
         <v>54</v>
       </c>
-      <c r="G8" s="0" t="s">
+      <c r="G8" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" t="s">
         <v>58</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" t="s">
         <v>59</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" t="s">
         <v>60</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="F9" t="s">
         <v>61</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" t="s">
         <v>63</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" t="s">
         <v>66</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" t="s">
         <v>67</v>
       </c>
-      <c r="F10" s="0" t="s">
+      <c r="F10" t="s">
         <v>68</v>
       </c>
-      <c r="G10" s="0" t="s">
+      <c r="G10" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" t="s">
         <v>72</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" t="s">
         <v>73</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" t="s">
         <v>74</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="F11" t="s">
         <v>75</v>
       </c>
-      <c r="G11" s="0" t="s">
+      <c r="G11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" t="s">
         <v>77</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" t="s">
         <v>78</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" t="s">
         <v>78</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" t="s">
         <v>79</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" t="s">
         <v>80</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="F12" t="s">
         <v>81</v>
       </c>
-      <c r="G12" s="0" t="s">
+      <c r="G12" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" t="s">
         <v>83</v>
       </c>
-      <c r="B13" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="D13" s="0" t="s">
+      <c r="B13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" t="s">
         <v>84</v>
       </c>
-      <c r="E13" s="0" t="s">
+      <c r="E13" t="s">
         <v>85</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="F13" t="s">
         <v>86</v>
       </c>
-      <c r="G13" s="0" t="s">
+      <c r="G13" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" t="s">
         <v>88</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" t="s">
         <v>89</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" t="s">
         <v>90</v>
       </c>
-      <c r="D14" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="E14" s="0" t="s">
+      <c r="D14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" t="s">
         <v>91</v>
       </c>
-      <c r="F14" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="G14" s="0" t="s">
+      <c r="F14" t="s">
+        <v>53</v>
+      </c>
+      <c r="G14" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" t="s">
         <v>93</v>
       </c>
-      <c r="B15" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="0" t="s">
+      <c r="B15" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" t="s">
         <v>89</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" t="s">
         <v>94</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" t="s">
         <v>95</v>
       </c>
-      <c r="F15" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="G15" s="0" t="s">
+      <c r="F15" t="s">
+        <v>53</v>
+      </c>
+      <c r="G15" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" t="s">
         <v>97</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" t="s">
         <v>89</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" t="s">
         <v>98</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" t="s">
         <v>99</v>
       </c>
-      <c r="E16" s="0" t="s">
+      <c r="E16" t="s">
         <v>100</v>
       </c>
-      <c r="F16" s="0" t="s">
+      <c r="F16" t="s">
         <v>101</v>
       </c>
-      <c r="G16" s="0" t="s">
+      <c r="G16" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" t="s">
         <v>103</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" t="s">
         <v>79</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" t="s">
         <v>104</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" t="s">
         <v>105</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="E17" t="s">
         <v>106</v>
       </c>
-      <c r="F17" s="0" t="s">
+      <c r="F17" t="s">
         <v>81</v>
       </c>
-      <c r="G17" s="0" t="s">
+      <c r="G17" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" t="s">
         <v>108</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" t="s">
         <v>84</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" t="s">
         <v>109</v>
       </c>
-      <c r="D18" s="0" t="s">
+      <c r="D18" t="s">
         <v>110</v>
       </c>
-      <c r="E18" s="0" t="s">
+      <c r="E18" t="s">
         <v>111</v>
       </c>
-      <c r="F18" s="0" t="s">
+      <c r="F18" t="s">
         <v>96</v>
       </c>
-      <c r="G18" s="0" t="s">
+      <c r="G18" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" t="s">
         <v>113</v>
       </c>
-      <c r="B19" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="0" t="s">
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" t="s">
         <v>98</v>
       </c>
-      <c r="D19" s="0" t="s">
+      <c r="D19" t="s">
         <v>114</v>
       </c>
-      <c r="E19" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="F19" s="0" t="s">
+      <c r="E19" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" t="s">
         <v>115</v>
       </c>
-      <c r="G19" s="0" t="s">
+      <c r="G19" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" t="s">
         <v>116</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" t="s">
         <v>89</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" t="s">
         <v>117</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="D20" t="s">
         <v>118</v>
       </c>
-      <c r="E20" s="0" t="s">
+      <c r="E20" t="s">
         <v>119</v>
       </c>
-      <c r="F20" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="G20" s="0" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="F20" t="s">
+        <v>53</v>
+      </c>
+      <c r="G20" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" t="s">
         <v>120</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" t="s">
         <v>106</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" t="s">
         <v>121</v>
       </c>
-      <c r="D21" s="0" t="s">
+      <c r="D21" t="s">
         <v>122</v>
       </c>
-      <c r="E21" s="0" t="s">
+      <c r="E21" t="s">
         <v>123</v>
       </c>
-      <c r="F21" s="0" t="s">
+      <c r="F21" t="s">
         <v>124</v>
       </c>
-      <c r="G21" s="0" t="s">
+      <c r="G21" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" t="s">
         <v>113</v>
       </c>
-      <c r="B22" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="C22" s="0" t="s">
+      <c r="B22" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" t="s">
         <v>98</v>
       </c>
-      <c r="D22" s="0" t="s">
+      <c r="D22" t="s">
         <v>114</v>
       </c>
-      <c r="E22" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="F22" s="0" t="s">
+      <c r="E22" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" t="s">
         <v>115</v>
       </c>
-      <c r="G22" s="0" t="s">
+      <c r="G22" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" ht="12.8" customHeight="1"/>
+    <row r="1048575" ht="12.8" customHeight="1"/>
+    <row r="1048576" ht="12.8" customHeight="1"/>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G1048576"/>
-  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" t="s">
         <v>126</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" t="s">
         <v>127</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" t="s">
         <v>128</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" t="s">
         <v>129</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" t="s">
         <v>130</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" t="s">
         <v>133</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" t="s">
         <v>134</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" t="s">
         <v>135</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" t="s">
         <v>136</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" t="s">
         <v>137</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" t="s">
         <v>37</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" t="s">
         <v>38</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" t="s">
         <v>39</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="F7" t="s">
         <v>40</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="G7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" ht="15" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>138</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" t="s">
         <v>139</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" t="s">
         <v>46</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="F9" t="s">
         <v>47</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" t="s">
         <v>140</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" t="s">
         <v>71</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" t="s">
         <v>72</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" t="s">
         <v>73</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" t="s">
         <v>74</v>
       </c>
-      <c r="F10" s="0" t="s">
+      <c r="F10" t="s">
         <v>75</v>
       </c>
-      <c r="G10" s="0" t="s">
+      <c r="G10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" t="s">
         <v>141</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" t="s">
         <v>52</v>
       </c>
-      <c r="E11" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="F11" s="0" t="s">
+      <c r="E11" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" t="s">
         <v>54</v>
       </c>
-      <c r="G11" s="0" t="s">
+      <c r="G11" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" t="s">
         <v>142</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" t="s">
         <v>57</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" t="s">
         <v>59</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" t="s">
         <v>60</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="F12" t="s">
         <v>61</v>
       </c>
-      <c r="G12" s="0" t="s">
+      <c r="G12" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" t="s">
         <v>143</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" t="s">
         <v>64</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" t="s">
         <v>65</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" t="s">
         <v>66</v>
       </c>
-      <c r="E13" s="0" t="s">
+      <c r="E13" t="s">
         <v>67</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="F13" t="s">
         <v>68</v>
       </c>
-      <c r="G13" s="0" t="s">
+      <c r="G13" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" ht="15" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>144</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" t="s">
         <v>145</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" t="s">
         <v>78</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" t="s">
         <v>78</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" t="s">
         <v>79</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" t="s">
         <v>80</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="F15" t="s">
         <v>81</v>
       </c>
-      <c r="G15" s="0" t="s">
+      <c r="G15" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" t="s">
         <v>146</v>
       </c>
-      <c r="B16" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="D16" s="0" t="s">
+      <c r="B16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16" t="s">
         <v>84</v>
       </c>
-      <c r="E16" s="0" t="s">
+      <c r="E16" t="s">
         <v>85</v>
       </c>
-      <c r="F16" s="0" t="s">
+      <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="G16" s="0" t="s">
+      <c r="G16" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" ht="15" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>147</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" t="s">
         <v>148</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" t="s">
         <v>89</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" t="s">
         <v>90</v>
       </c>
-      <c r="D18" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="E18" s="0" t="s">
+      <c r="D18" t="s">
+        <v>53</v>
+      </c>
+      <c r="E18" t="s">
         <v>91</v>
       </c>
-      <c r="F18" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="G18" s="0" t="s">
+      <c r="F18" t="s">
+        <v>53</v>
+      </c>
+      <c r="G18" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" t="s">
         <v>149</v>
       </c>
-      <c r="B19" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="0" t="s">
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" t="s">
         <v>89</v>
       </c>
-      <c r="D19" s="0" t="s">
+      <c r="D19" t="s">
         <v>94</v>
       </c>
-      <c r="E19" s="0" t="s">
+      <c r="E19" t="s">
         <v>95</v>
       </c>
-      <c r="F19" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="G19" s="0" t="s">
+      <c r="F19" t="s">
+        <v>53</v>
+      </c>
+      <c r="G19" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" t="s">
         <v>150</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" t="s">
         <v>89</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" t="s">
         <v>98</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="D20" t="s">
         <v>99</v>
       </c>
-      <c r="E20" s="0" t="s">
+      <c r="E20" t="s">
         <v>100</v>
       </c>
-      <c r="F20" s="0" t="s">
+      <c r="F20" t="s">
         <v>101</v>
       </c>
-      <c r="G20" s="0" t="s">
+      <c r="G20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" t="s">
         <v>151</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" t="s">
         <v>79</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" t="s">
         <v>104</v>
       </c>
-      <c r="D21" s="0" t="s">
+      <c r="D21" t="s">
         <v>105</v>
       </c>
-      <c r="E21" s="0" t="s">
+      <c r="E21" t="s">
         <v>106</v>
       </c>
-      <c r="F21" s="0" t="s">
+      <c r="F21" t="s">
         <v>81</v>
       </c>
-      <c r="G21" s="0" t="s">
+      <c r="G21" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" t="s">
         <v>152</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" t="s">
         <v>84</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" t="s">
         <v>109</v>
       </c>
-      <c r="D22" s="0" t="s">
+      <c r="D22" t="s">
         <v>110</v>
       </c>
-      <c r="E22" s="0" t="s">
+      <c r="E22" t="s">
         <v>111</v>
       </c>
-      <c r="F22" s="0" t="s">
+      <c r="F22" t="s">
         <v>96</v>
       </c>
-      <c r="G22" s="0" t="s">
+      <c r="G22" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" t="s">
         <v>153</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" t="s">
         <v>89</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="C23" t="s">
         <v>117</v>
       </c>
-      <c r="D23" s="0" t="s">
+      <c r="D23" t="s">
         <v>118</v>
       </c>
-      <c r="E23" s="0" t="s">
+      <c r="E23" t="s">
         <v>119</v>
       </c>
-      <c r="F23" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="G23" s="0" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="F23" t="s">
+        <v>53</v>
+      </c>
+      <c r="G23" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" t="s">
         <v>154</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" t="s">
         <v>106</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="C24" t="s">
         <v>121</v>
       </c>
-      <c r="D24" s="0" t="s">
+      <c r="D24" t="s">
         <v>122</v>
       </c>
-      <c r="E24" s="0" t="s">
+      <c r="E24" t="s">
         <v>123</v>
       </c>
-      <c r="F24" s="0" t="s">
+      <c r="F24" t="s">
         <v>124</v>
       </c>
-      <c r="G24" s="0" t="s">
+      <c r="G24" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" t="s">
         <v>155</v>
       </c>
-      <c r="B25" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="C25" s="0" t="s">
+      <c r="B25" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" t="s">
         <v>98</v>
       </c>
-      <c r="D25" s="0" t="s">
+      <c r="D25" t="s">
         <v>114</v>
       </c>
-      <c r="E25" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="F25" s="0" t="s">
+      <c r="E25" t="s">
+        <v>53</v>
+      </c>
+      <c r="F25" t="s">
         <v>115</v>
       </c>
-      <c r="G25" s="0" t="s">
+      <c r="G25" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" ht="12.8" customHeight="1"/>
+    <row r="1048574" ht="12.8" customHeight="1"/>
+    <row r="1048575" ht="12.8" customHeight="1"/>
+    <row r="1048576" ht="12.8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:C2"/>
@@ -1825,12 +1773,11 @@
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A17:C17"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.511805555555556" right="0.511805555555556" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
May: rodando tabela nova
</commit_message>
<xml_diff>
--- a/tabela de habitat.xlsx
+++ b/tabela de habitat.xlsx
@@ -1,21 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="tabela_final" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="tabela_final" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <extLst>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="156">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
@@ -488,11 +494,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -501,10 +507,26 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -516,7 +538,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -524,20 +546,49 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment textRotation="0" horizontal="left" vertical="bottom" indent="0"/>
-      <protection hidden="0" locked="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
 </styleSheet>
 </file>
 
@@ -717,1055 +768,1056 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <dimension ref="A1:G1048576"/>
+  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
-      <c r="A1" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="0" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
-      <c r="A2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="0" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1">
-      <c r="A3" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="0" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
-      <c r="A4" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="0" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="0" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
         <v>42</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="0" t="s">
         <v>44</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="0" t="s">
         <v>46</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="0" t="s">
         <v>47</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
         <v>49</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="0" t="s">
         <v>51</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="E8" t="s">
-        <v>53</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="E8" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="0" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="0" t="s">
         <v>57</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="0" t="s">
         <v>60</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="0" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
         <v>63</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="0" t="s">
         <v>64</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="0" t="s">
         <v>65</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="0" t="s">
         <v>67</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="0" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="0" t="s">
         <v>72</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="0" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="A12" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
         <v>77</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="0" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="A13" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="B13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" t="s">
-        <v>53</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="B13" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="0" t="s">
         <v>86</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="0" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
         <v>88</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="D14" t="s">
-        <v>53</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="D14" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="F14" t="s">
-        <v>53</v>
-      </c>
-      <c r="G14" t="s">
+      <c r="F14" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="G14" s="0" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="B15" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="B15" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="F15" t="s">
-        <v>53</v>
-      </c>
-      <c r="G15" t="s">
+      <c r="F15" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="G15" s="0" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
         <v>97</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="0" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
         <v>103</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="0" t="s">
         <v>104</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="0" t="s">
         <v>106</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="0" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
         <v>108</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="0" t="s">
         <v>109</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="0" t="s">
         <v>110</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="0" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
         <v>113</v>
       </c>
-      <c r="B19" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="B19" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="0" t="s">
         <v>114</v>
       </c>
-      <c r="E19" t="s">
-        <v>53</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="E19" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="0" t="s">
         <v>115</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="0" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
         <v>116</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="0" t="s">
         <v>117</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="0" t="s">
         <v>118</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="0" t="s">
         <v>119</v>
       </c>
-      <c r="F20" t="s">
-        <v>53</v>
-      </c>
-      <c r="G20" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" t="s">
+      <c r="F20" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="G20" s="0" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
         <v>120</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="0" t="s">
         <v>106</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="0" t="s">
         <v>121</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="0" t="s">
         <v>122</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="0" t="s">
         <v>123</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="0" t="s">
         <v>124</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="0" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1">
-      <c r="A22" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
         <v>113</v>
       </c>
-      <c r="B22" t="s">
-        <v>53</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="B22" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="0" t="s">
         <v>114</v>
       </c>
-      <c r="E22" t="s">
-        <v>53</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="E22" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" s="0" t="s">
         <v>115</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22" s="0" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="1048574" ht="12.8" customHeight="1"/>
-    <row r="1048575" ht="12.8" customHeight="1"/>
-    <row r="1048576" ht="12.8" customHeight="1"/>
+    <row r="1048574" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.597222222222222" bottom="0.597222222222222" header="0.511805555555556" footer="0.511805555555556"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
-    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
-    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <dimension ref="A1:G1048576"/>
+  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
-      <c r="A1" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="0" t="s">
         <v>126</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="0" t="s">
         <v>127</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="0" t="s">
         <v>128</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="0" t="s">
         <v>129</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="0" t="s">
         <v>130</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="0" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" ht="15" customHeight="1">
-      <c r="A3" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
         <v>133</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="0" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
-      <c r="A4" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="0" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
         <v>136</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="0" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
         <v>137</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="0" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>138</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
     </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
         <v>139</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="0" t="s">
         <v>44</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="0" t="s">
         <v>46</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="0" t="s">
         <v>47</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
         <v>140</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="0" t="s">
         <v>72</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="0" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
         <v>141</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="0" t="s">
         <v>51</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="E11" t="s">
-        <v>53</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="E11" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="0" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="A12" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
         <v>142</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="0" t="s">
         <v>57</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="0" t="s">
         <v>60</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="0" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="A13" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
         <v>143</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="0" t="s">
         <v>64</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="0" t="s">
         <v>65</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="0" t="s">
         <v>67</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="0" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>144</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
     </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
         <v>145</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="0" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
         <v>146</v>
       </c>
-      <c r="B16" t="s">
-        <v>53</v>
-      </c>
-      <c r="C16" t="s">
-        <v>53</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="B16" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="0" t="s">
         <v>86</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="0" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
         <v>147</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
         <v>148</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="D18" t="s">
-        <v>53</v>
-      </c>
-      <c r="E18" t="s">
+      <c r="D18" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E18" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="F18" t="s">
-        <v>53</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="F18" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="G18" s="0" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
         <v>149</v>
       </c>
-      <c r="B19" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="B19" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="F19" t="s">
-        <v>53</v>
-      </c>
-      <c r="G19" t="s">
+      <c r="F19" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="G19" s="0" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
         <v>150</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="0" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
         <v>151</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="0" t="s">
         <v>104</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="0" t="s">
         <v>106</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="0" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1">
-      <c r="A22" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
         <v>152</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="0" t="s">
         <v>109</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="0" t="s">
         <v>110</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22" s="0" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="A23" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="s">
         <v>153</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="0" t="s">
         <v>117</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="0" t="s">
         <v>118</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="0" t="s">
         <v>119</v>
       </c>
-      <c r="F23" t="s">
-        <v>53</v>
-      </c>
-      <c r="G23" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1">
-      <c r="A24" t="s">
+      <c r="F23" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="G23" s="0" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="s">
         <v>154</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="0" t="s">
         <v>106</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="0" t="s">
         <v>121</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="0" t="s">
         <v>122</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="0" t="s">
         <v>123</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="0" t="s">
         <v>124</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" s="0" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1">
-      <c r="A25" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
         <v>155</v>
       </c>
-      <c r="B25" t="s">
-        <v>53</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="B25" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="0" t="s">
         <v>114</v>
       </c>
-      <c r="E25" t="s">
-        <v>53</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="E25" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="F25" s="0" t="s">
         <v>115</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="0" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="1048573" ht="12.8" customHeight="1"/>
-    <row r="1048574" ht="12.8" customHeight="1"/>
-    <row r="1048575" ht="12.8" customHeight="1"/>
-    <row r="1048576" ht="12.8" customHeight="1"/>
+    <row r="1048573" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:C2"/>
@@ -1773,11 +1825,12 @@
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A17:C17"/>
   </mergeCells>
-  <pageMargins left="0.511805555555556" right="0.511805555555556" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.511805555555556" right="0.511805555555556" top="0.634722222222222" bottom="0.634722222222222" header="0.511805555555556" footer="0.511805555555556"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
-    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
-    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>